<commit_message>
Stand 31.07.2026: Einbau Patch 18 (Agenda Centre of Gravity) + Verifikation
</commit_message>
<xml_diff>
--- a/results/empirics/goldstandard/goldstandard_v2_carried.xlsx
+++ b/results/empirics/goldstandard/goldstandard_v2_carried.xlsx
@@ -4636,7 +4636,7 @@
         <v>57</v>
       </c>
       <c r="L5" t="n">
-        <v>0.682414174079895</v>
+        <v>0.682422637939453</v>
       </c>
       <c r="M5" t="s">
         <v>47</v>
@@ -6152,7 +6152,7 @@
         <v>117</v>
       </c>
       <c r="L28" t="n">
-        <v>0.44936329126358</v>
+        <v>0.45016023516655</v>
       </c>
       <c r="M28" t="s">
         <v>63</v>
@@ -8316,7 +8316,7 @@
         <v>231</v>
       </c>
       <c r="L61" t="n">
-        <v>0.394578725099564</v>
+        <v>0.395102024078369</v>
       </c>
       <c r="M61" t="s">
         <v>85</v>
@@ -16504,7 +16504,7 @@
         <v>143</v>
       </c>
       <c r="L186" t="n">
-        <v>0.337611049413681</v>
+        <v>0.336877644062042</v>
       </c>
       <c r="M186" t="s">
         <v>63</v>
@@ -18792,7 +18792,7 @@
         <v>84</v>
       </c>
       <c r="L221" t="n">
-        <v>0.974586009979248</v>
+        <v>0.974580824375153</v>
       </c>
       <c r="M221" t="s">
         <v>85</v>

</xml_diff>